<commit_message>
Rebuild site from client documents: 12 pages, design.md, Telegram
- content/: факты только из прайса, регламента и договора (Архив/, вне git);
  prices.json — единственное место цен, пробелы — content/probely.md
- 12 страниц по карте: главная, услуги ×6, цены, запись, гарантия и оплата, вопросы;
  меню и sitemap.xml из одного списка PAGES в scripts/build.mjs
- design.md: 2 цвета + нейтральный, один шрифт Manrope, карточка услуги, кнопка
- CLAUDE.md v2: 5 главных правил
- запись по режиму работы из регламента, ?usluga= выбирает услугу в форме
- сборка падает на «от N», отзывах, сроках работ и токене бота в n8n/ и js/
- vercel.json: сборка в dist/ и заголовки безопасности; наружу только dist/
- n8n: проверка записи по режиму работы, уведомления в Telegram
  (заглушки BOT_TOKEN_TG и CHAT_ID_TG)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/n8n/shesterenka-leads-template.xlsx
+++ b/n8n/shesterenka-leads-template.xlsx
@@ -469,15 +469,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" style="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -498,31 +500,41 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Услуга</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>Что случилось</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Запись</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Время</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:F1000">
+  <conditionalFormatting sqref="A2:H1000">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$F2="Новая"</formula>
+      <formula>$H2="Новая"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$F2="Отказ"</formula>
+      <formula>$H2="Отказ"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Статус" error="Выберите статус из списка" type="list">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Статус" error="Выберите статус из списка" type="list">
       <formula1>"Новая,Перезвонили,Записан,Отказ"</formula1>
     </dataValidation>
   </dataValidations>
@@ -536,15 +548,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,81 +619,125 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Время</t>
+          <t>Услуга</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Время приёма заявки сервером n8n, по Москве.</t>
+          <t>Услуга, выбранная в форме. Пусто — клиенту нужна консультация.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Запись</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Желаемые день и время визита. Пусто — клиент не выбрал. Запись предварительная: подтвердите время по телефону.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Время</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Время приёма заявки сервером n8n, по Москве.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Пример строки (так её запишет n8n)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Имя</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Телефон</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Марка</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Услуга</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Что случилось</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Запись</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Время</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Иван</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>+79161234567</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Kia Rio 2018</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Ходовая часть</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Стучит спереди справа на кочках</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>09.10.2026, 14:30:47</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>21.10.2026 10:00</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>19.10.2026, 14:30:47</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Новая</t>
         </is>

</xml_diff>